<commit_message>
Improve cleaning worksheet with callback and credit reconciliation [skip social]
</commit_message>
<xml_diff>
--- a/public/downloads/mybreakeven-cleaning-job-cost.xlsx
+++ b/public/downloads/mybreakeven-cleaning-job-cost.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job" sheetId="1" r:id="R5b2f3fcdc73e4ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="2" r:id="Rae68ff4fac524359"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job" sheetId="1" r:id="R0ac3e104fdd3472d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="2" r:id="Rf406422c6b014f6e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -99,7 +99,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -115,6 +115,17 @@
     <x:xf numFmtId="202" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -361,7 +372,7 @@
     </x:row>
     <x:row r="3" ht="31" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Enter every input, including zero when a cost does not apply</x:v>
+        <x:v>Enter first-visit actuals; add adjustments below</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -381,19 +392,19 @@
         <x:v>Actual minus estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="1" t="str">
+    <x:row r="5" ht="48" customHeight="1">
+      <x:c r="A5" s="15" t="str">
         <x:v>Contribution before monthly overhead</x:v>
       </x:c>
-      <x:c r="B5" s="6" t="str">
+      <x:c r="B5" s="16" t="str">
         <x:f>B26</x:f>
         <x:v>Enter all inputs</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="str">
-        <x:f>C26</x:f>
-        <x:v>Enter all inputs</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="str">
+      <x:c r="C5" s="16" t="str">
+        <x:f>C51</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="str">
         <x:f>IF(AND(ISNUMBER(B5),ISNUMBER(C5)),C5-B5,"Complete both columns")</x:f>
         <x:v>Complete both columns</x:v>
       </x:c>
@@ -406,7 +417,7 @@
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="1" t="str">
-        <x:v>A lower contribution difference means less left for overhead.</x:v>
+        <x:v>Actual result includes adjustments below; costs entered once.</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -551,7 +562,7 @@
         <x:v>Enter all inputs</x:v>
       </x:c>
       <x:c r="C23" s="6" t="str">
-        <x:f>IF(COUNT(C12:C18)=7,C12*C18,"Enter all inputs")</x:f>
+        <x:f>IF(COUNT(C12:C18)=7,IF(ISNUMBER(C43),C43,C12*C18),"Enter all inputs")</x:f>
         <x:v>Enter all inputs</x:v>
       </x:c>
       <x:c r="D23" s="1"/>
@@ -652,11 +663,347 @@
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>Example source: MyBreakeven illustrative assumptions, October 10, 2026.</x:v>
+        <x:v>Example source: MyBreakeven illustrative assumptions, October 14, 2026.</x:v>
       </x:c>
       <x:c r="B34" s="14"/>
       <x:c r="C34" s="14"/>
       <x:c r="D34" s="14"/>
+    </x:row>
+    <x:row r="36" ht="30" customHeight="1">
+      <x:c r="A36" s="8" t="str">
+        <x:v>Additional actual job entries</x:v>
+      </x:c>
+      <x:c r="B36" s="8"/>
+      <x:c r="C36" s="8"/>
+      <x:c r="D36" s="1"/>
+    </x:row>
+    <x:row r="37" ht="25" customHeight="1">
+      <x:c r="A37" s="1" t="str">
+        <x:v>Callback paid crew-hours</x:v>
+      </x:c>
+      <x:c r="B37" s="1"/>
+      <x:c r="C37" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D37" s="1"/>
+    </x:row>
+    <x:row r="38" ht="25" customHeight="1">
+      <x:c r="A38" s="1" t="str">
+        <x:v>Callback loaded cost per crew-hour</x:v>
+      </x:c>
+      <x:c r="B38" s="1"/>
+      <x:c r="C38" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="25" customHeight="1">
+      <x:c r="A39" s="1" t="str">
+        <x:v>Callback supplies</x:v>
+      </x:c>
+      <x:c r="B39" s="1"/>
+      <x:c r="C39" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="25" customHeight="1">
+      <x:c r="A40" s="1" t="str">
+        <x:v>Callback travel</x:v>
+      </x:c>
+      <x:c r="B40" s="1"/>
+      <x:c r="C40" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="25" customHeight="1">
+      <x:c r="A41" s="1" t="str">
+        <x:v>Callback other direct costs</x:v>
+      </x:c>
+      <x:c r="B41" s="1"/>
+      <x:c r="C41" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="25" customHeight="1">
+      <x:c r="A42" s="1" t="str">
+        <x:v>Customer credit / revenue reduction</x:v>
+      </x:c>
+      <x:c r="B42" s="1"/>
+      <x:c r="C42" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="25" customHeight="1">
+      <x:c r="A43" s="1" t="str">
+        <x:v>Actual payment fees (optional override)</x:v>
+      </x:c>
+      <x:c r="B43" s="1"/>
+      <x:c r="C43" s="11"/>
+      <x:c r="D43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="25" customHeight="1">
+      <x:c r="A44" s="1" t="str">
+        <x:v>Extra work revenue</x:v>
+      </x:c>
+      <x:c r="B44" s="1"/>
+      <x:c r="C44" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D44" s="1"/>
+    </x:row>
+    <x:row r="45" ht="25" customHeight="1">
+      <x:c r="A45" s="1" t="str">
+        <x:v>Extra work variable costs</x:v>
+      </x:c>
+      <x:c r="B45" s="1"/>
+      <x:c r="C45" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D45" s="1"/>
+    </x:row>
+    <x:row r="46" ht="25" customHeight="1">
+      <x:c r="A46" s="1"/>
+      <x:c r="B46" s="1"/>
+      <x:c r="C46" s="1"/>
+      <x:c r="D46" s="1"/>
+    </x:row>
+    <x:row r="47" ht="30" customHeight="1">
+      <x:c r="A47" s="8" t="str">
+        <x:v>Final job result</x:v>
+      </x:c>
+      <x:c r="B47" s="8"/>
+      <x:c r="C47" s="8"/>
+      <x:c r="D47" s="1"/>
+    </x:row>
+    <x:row r="48" ht="25" customHeight="1">
+      <x:c r="A48" s="1" t="str">
+        <x:v>Callback cost</x:v>
+      </x:c>
+      <x:c r="B48" s="1"/>
+      <x:c r="C48" s="6" t="n">
+        <x:f>IF(COUNT(C37:C42,C44:C45)=8,C37*C38+SUM(C39:C41),"Enter every adjustment")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D48" s="1"/>
+    </x:row>
+    <x:row r="49" ht="25" customHeight="1">
+      <x:c r="A49" s="1" t="str">
+        <x:v>Final retained revenue</x:v>
+      </x:c>
+      <x:c r="B49" s="1"/>
+      <x:c r="C49" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(C26),ISNUMBER(C48)),C12-C42+C44,"Complete actual and adjustments")</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D49" s="1"/>
+    </x:row>
+    <x:row r="50" ht="25" customHeight="1">
+      <x:c r="A50" s="1" t="str">
+        <x:v>Total variable costs incl. adjustments</x:v>
+      </x:c>
+      <x:c r="B50" s="1"/>
+      <x:c r="C50" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(C24),ISNUMBER(C48)),C24+C48+C45,"Complete actual and adjustments")</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D50" s="1"/>
+    </x:row>
+    <x:row r="51" ht="25" customHeight="1">
+      <x:c r="A51" s="1" t="str">
+        <x:v>Final contribution before overhead</x:v>
+      </x:c>
+      <x:c r="B51" s="1"/>
+      <x:c r="C51" s="17" t="str">
+        <x:f>IF(AND(ISNUMBER(C49),ISNUMBER(C50)),C49-C50,"Complete actual and adjustments")</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D51" s="1"/>
+    </x:row>
+    <x:row r="52" ht="25" customHeight="1">
+      <x:c r="A52" s="1" t="str">
+        <x:v>Contribution / retained revenue</x:v>
+      </x:c>
+      <x:c r="B52" s="1"/>
+      <x:c r="C52" s="18" t="str">
+        <x:f>IF(AND(ISNUMBER(C51),ISNUMBER(C49)),IF(C49=0,"n.a.",C51/C49),"Complete actual and adjustments")</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D52" s="1"/>
+    </x:row>
+    <x:row r="53" ht="25" customHeight="1">
+      <x:c r="A53" s="1" t="str">
+        <x:v>Final actual minus estimate</x:v>
+      </x:c>
+      <x:c r="B53" s="1"/>
+      <x:c r="C53" s="17" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C51-B26,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D53" s="1"/>
+    </x:row>
+    <x:row r="54" ht="25" customHeight="1">
+      <x:c r="A54" s="1"/>
+      <x:c r="B54" s="1"/>
+      <x:c r="C54" s="1"/>
+      <x:c r="D54" s="1"/>
+    </x:row>
+    <x:row r="55" ht="25" customHeight="1">
+      <x:c r="A55" s="1"/>
+      <x:c r="B55" s="1"/>
+      <x:c r="C55" s="1"/>
+      <x:c r="D55" s="1"/>
+    </x:row>
+    <x:row r="56" ht="25" customHeight="1">
+      <x:c r="A56" s="1"/>
+      <x:c r="B56" s="1"/>
+      <x:c r="C56" s="1"/>
+      <x:c r="D56" s="1"/>
+    </x:row>
+    <x:row r="57" ht="30" customHeight="1">
+      <x:c r="A57" s="8" t="str">
+        <x:v>Contribution change by driver</x:v>
+      </x:c>
+      <x:c r="B57" s="8"/>
+      <x:c r="C57" s="8"/>
+      <x:c r="D57" s="1"/>
+    </x:row>
+    <x:row r="58" ht="25" customHeight="1">
+      <x:c r="A58" s="1" t="str">
+        <x:v>First-visit revenue</x:v>
+      </x:c>
+      <x:c r="B58" s="1"/>
+      <x:c r="C58" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C12-B12,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D58" s="1"/>
+    </x:row>
+    <x:row r="59" ht="25" customHeight="1">
+      <x:c r="A59" s="1" t="str">
+        <x:v>First-visit labour</x:v>
+      </x:c>
+      <x:c r="B59" s="1"/>
+      <x:c r="C59" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B22-C22,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D59" s="1"/>
+    </x:row>
+    <x:row r="60" ht="25" customHeight="1">
+      <x:c r="A60" s="1" t="str">
+        <x:v>First-visit supplies</x:v>
+      </x:c>
+      <x:c r="B60" s="1"/>
+      <x:c r="C60" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B15-C15,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D60" s="1"/>
+    </x:row>
+    <x:row r="61" ht="25" customHeight="1">
+      <x:c r="A61" s="1" t="str">
+        <x:v>First-visit travel</x:v>
+      </x:c>
+      <x:c r="B61" s="1"/>
+      <x:c r="C61" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B16-C16,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D61" s="1"/>
+    </x:row>
+    <x:row r="62" ht="25" customHeight="1">
+      <x:c r="A62" s="1" t="str">
+        <x:v>First-visit other direct costs</x:v>
+      </x:c>
+      <x:c r="B62" s="1"/>
+      <x:c r="C62" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B17-C17,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D62" s="1"/>
+    </x:row>
+    <x:row r="63" ht="25" customHeight="1">
+      <x:c r="A63" s="1" t="str">
+        <x:v>Payment fees</x:v>
+      </x:c>
+      <x:c r="B63" s="1"/>
+      <x:c r="C63" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B23-C23,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D63" s="1"/>
+    </x:row>
+    <x:row r="64" ht="25" customHeight="1">
+      <x:c r="A64" s="1" t="str">
+        <x:v>Callback</x:v>
+      </x:c>
+      <x:c r="B64" s="1"/>
+      <x:c r="C64" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),-C48,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D64" s="1"/>
+    </x:row>
+    <x:row r="65" ht="25" customHeight="1">
+      <x:c r="A65" s="1" t="str">
+        <x:v>Customer credit</x:v>
+      </x:c>
+      <x:c r="B65" s="1"/>
+      <x:c r="C65" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),-C42,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D65" s="1"/>
+    </x:row>
+    <x:row r="66" ht="25" customHeight="1">
+      <x:c r="A66" s="1" t="str">
+        <x:v>Extra work net contribution</x:v>
+      </x:c>
+      <x:c r="B66" s="1"/>
+      <x:c r="C66" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C44-C45,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D66" s="1"/>
+    </x:row>
+    <x:row r="67" ht="25" customHeight="1">
+      <x:c r="A67" s="1" t="str">
+        <x:v>Total contribution change</x:v>
+      </x:c>
+      <x:c r="B67" s="1"/>
+      <x:c r="C67" s="6" t="str">
+        <x:f>IF(COUNT(C58:C66)=9,SUM(C58:C66),"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D67" s="1"/>
+    </x:row>
+    <x:row r="68" ht="48" customHeight="1">
+      <x:c r="A68" s="19" t="str">
+        <x:v>Enter callback and extra costs only when absent from first-visit actuals. Credit reduces revenue once.</x:v>
+      </x:c>
+      <x:c r="B68" s="1"/>
+      <x:c r="C68" s="1"/>
+      <x:c r="D68" s="1"/>
+    </x:row>
+    <x:row r="69" ht="48" customHeight="1">
+      <x:c r="A69" s="19" t="str">
+        <x:v>Blank fee override uses first-visit revenue × rate. Include extra-work fees once in override or extra costs.</x:v>
+      </x:c>
+      <x:c r="B69" s="1"/>
+      <x:c r="C69" s="1"/>
+      <x:c r="D69" s="1"/>
+    </x:row>
+    <x:row r="70" ht="48" customHeight="1">
+      <x:c r="A70" s="19" t="str">
+        <x:v>All figures use one currency. Contribution excludes fixed overhead. Example is fictional.</x:v>
+      </x:c>
+      <x:c r="B70" s="1"/>
+      <x:c r="C70" s="1"/>
+      <x:c r="D70" s="1"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="D5:D5">
@@ -664,7 +1011,7 @@
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="decimal" operator="between" sqref="B12:C17">
       <x:formula1>0</x:formula1>
       <x:formula2>1000000000</x:formula2>
@@ -672,6 +1019,10 @@
     <x:dataValidation type="decimal" operator="between" sqref="B18:C18">
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="C37:C45">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1000000000</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -704,7 +1055,7 @@
     </x:row>
     <x:row r="3" ht="31" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Illustrative USD example, not a customer result</x:v>
+        <x:v>Fictional USD job including callback and credit</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -724,21 +1075,21 @@
         <x:v>Actual minus estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="1" t="str">
+    <x:row r="5" ht="48" customHeight="1">
+      <x:c r="A5" s="15" t="str">
         <x:v>Contribution before monthly overhead</x:v>
       </x:c>
-      <x:c r="B5" s="6" t="n">
+      <x:c r="B5" s="16" t="n">
         <x:f>B26</x:f>
         <x:v>110.80000000000001</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="n">
-        <x:f>C26</x:f>
-        <x:v>78.80000000000001</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="n">
+      <x:c r="C5" s="16" t="n">
+        <x:f>C51</x:f>
+        <x:v>21.80000000000001</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="n">
         <x:f>IF(AND(ISNUMBER(B5),ISNUMBER(C5)),C5-B5,"Complete both columns")</x:f>
-        <x:v>-32</x:v>
+        <x:v>-89</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
@@ -749,7 +1100,7 @@
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="1" t="str">
-        <x:v>A lower contribution difference means less left for overhead.</x:v>
+        <x:v>Actual result includes adjustments below; costs entered once.</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -926,8 +1277,8 @@
         <x:v>7.199999999999999</x:v>
       </x:c>
       <x:c r="C23" s="6" t="n">
-        <x:f>IF(COUNT(C12:C18)=7,C12*C18,"Enter all inputs")</x:f>
-        <x:v>7.199999999999999</x:v>
+        <x:f>IF(COUNT(C12:C18)=7,IF(ISNUMBER(C43),C43,C12*C18),"Enter all inputs")</x:f>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="D23" s="1"/>
     </x:row>
@@ -1027,11 +1378,349 @@
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>Example source: MyBreakeven illustrative assumptions, October 10, 2026.</x:v>
+        <x:v>Example source: MyBreakeven illustrative assumptions, October 14, 2026.</x:v>
       </x:c>
       <x:c r="B34" s="14"/>
       <x:c r="C34" s="14"/>
       <x:c r="D34" s="14"/>
+    </x:row>
+    <x:row r="36" ht="30" customHeight="1">
+      <x:c r="A36" s="8" t="str">
+        <x:v>Additional actual job entries</x:v>
+      </x:c>
+      <x:c r="B36" s="8"/>
+      <x:c r="C36" s="8"/>
+      <x:c r="D36" s="1"/>
+    </x:row>
+    <x:row r="37" ht="25" customHeight="1">
+      <x:c r="A37" s="1" t="str">
+        <x:v>Callback paid crew-hours</x:v>
+      </x:c>
+      <x:c r="B37" s="1"/>
+      <x:c r="C37" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D37" s="1"/>
+    </x:row>
+    <x:row r="38" ht="25" customHeight="1">
+      <x:c r="A38" s="1" t="str">
+        <x:v>Callback loaded cost per crew-hour</x:v>
+      </x:c>
+      <x:c r="B38" s="1"/>
+      <x:c r="C38" s="11" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="25" customHeight="1">
+      <x:c r="A39" s="1" t="str">
+        <x:v>Callback supplies</x:v>
+      </x:c>
+      <x:c r="B39" s="1"/>
+      <x:c r="C39" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="25" customHeight="1">
+      <x:c r="A40" s="1" t="str">
+        <x:v>Callback travel</x:v>
+      </x:c>
+      <x:c r="B40" s="1"/>
+      <x:c r="C40" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="25" customHeight="1">
+      <x:c r="A41" s="1" t="str">
+        <x:v>Callback other direct costs</x:v>
+      </x:c>
+      <x:c r="B41" s="1"/>
+      <x:c r="C41" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="25" customHeight="1">
+      <x:c r="A42" s="1" t="str">
+        <x:v>Customer credit / revenue reduction</x:v>
+      </x:c>
+      <x:c r="B42" s="1"/>
+      <x:c r="C42" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="25" customHeight="1">
+      <x:c r="A43" s="1" t="str">
+        <x:v>Actual payment fees (optional override)</x:v>
+      </x:c>
+      <x:c r="B43" s="1"/>
+      <x:c r="C43" s="11" t="n">
+        <x:v>7.2</x:v>
+      </x:c>
+      <x:c r="D43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="25" customHeight="1">
+      <x:c r="A44" s="1" t="str">
+        <x:v>Extra work revenue</x:v>
+      </x:c>
+      <x:c r="B44" s="1"/>
+      <x:c r="C44" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D44" s="1"/>
+    </x:row>
+    <x:row r="45" ht="25" customHeight="1">
+      <x:c r="A45" s="1" t="str">
+        <x:v>Extra work variable costs</x:v>
+      </x:c>
+      <x:c r="B45" s="1"/>
+      <x:c r="C45" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D45" s="1"/>
+    </x:row>
+    <x:row r="46" ht="25" customHeight="1">
+      <x:c r="A46" s="1"/>
+      <x:c r="B46" s="1"/>
+      <x:c r="C46" s="1"/>
+      <x:c r="D46" s="1"/>
+    </x:row>
+    <x:row r="47" ht="30" customHeight="1">
+      <x:c r="A47" s="8" t="str">
+        <x:v>Final job result</x:v>
+      </x:c>
+      <x:c r="B47" s="8"/>
+      <x:c r="C47" s="8"/>
+      <x:c r="D47" s="1"/>
+    </x:row>
+    <x:row r="48" ht="25" customHeight="1">
+      <x:c r="A48" s="1" t="str">
+        <x:v>Callback cost</x:v>
+      </x:c>
+      <x:c r="B48" s="1"/>
+      <x:c r="C48" s="6" t="n">
+        <x:f>IF(COUNT(C37:C42,C44:C45)=8,C37*C38+SUM(C39:C41),"Enter every adjustment")</x:f>
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="D48" s="1"/>
+    </x:row>
+    <x:row r="49" ht="25" customHeight="1">
+      <x:c r="A49" s="1" t="str">
+        <x:v>Final retained revenue</x:v>
+      </x:c>
+      <x:c r="B49" s="1"/>
+      <x:c r="C49" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(C26),ISNUMBER(C48)),C12-C42+C44,"Complete actual and adjustments")</x:f>
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="D49" s="1"/>
+    </x:row>
+    <x:row r="50" ht="25" customHeight="1">
+      <x:c r="A50" s="1" t="str">
+        <x:v>Total variable costs incl. adjustments</x:v>
+      </x:c>
+      <x:c r="B50" s="1"/>
+      <x:c r="C50" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(C24),ISNUMBER(C48)),C24+C48+C45,"Complete actual and adjustments")</x:f>
+        <x:v>198.2</x:v>
+      </x:c>
+      <x:c r="D50" s="1"/>
+    </x:row>
+    <x:row r="51" ht="25" customHeight="1">
+      <x:c r="A51" s="1" t="str">
+        <x:v>Final contribution before overhead</x:v>
+      </x:c>
+      <x:c r="B51" s="1"/>
+      <x:c r="C51" s="17" t="n">
+        <x:f>IF(AND(ISNUMBER(C49),ISNUMBER(C50)),C49-C50,"Complete actual and adjustments")</x:f>
+        <x:v>21.80000000000001</x:v>
+      </x:c>
+      <x:c r="D51" s="1"/>
+    </x:row>
+    <x:row r="52" ht="25" customHeight="1">
+      <x:c r="A52" s="1" t="str">
+        <x:v>Contribution / retained revenue</x:v>
+      </x:c>
+      <x:c r="B52" s="1"/>
+      <x:c r="C52" s="18" t="n">
+        <x:f>IF(AND(ISNUMBER(C51),ISNUMBER(C49)),IF(C49=0,"n.a.",C51/C49),"Complete actual and adjustments")</x:f>
+        <x:v>0.09909090909090915</x:v>
+      </x:c>
+      <x:c r="D52" s="1"/>
+    </x:row>
+    <x:row r="53" ht="25" customHeight="1">
+      <x:c r="A53" s="1" t="str">
+        <x:v>Final actual minus estimate</x:v>
+      </x:c>
+      <x:c r="B53" s="1"/>
+      <x:c r="C53" s="17" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C51-B26,"Complete both columns")</x:f>
+        <x:v>-89</x:v>
+      </x:c>
+      <x:c r="D53" s="1"/>
+    </x:row>
+    <x:row r="54" ht="25" customHeight="1">
+      <x:c r="A54" s="1"/>
+      <x:c r="B54" s="1"/>
+      <x:c r="C54" s="1"/>
+      <x:c r="D54" s="1"/>
+    </x:row>
+    <x:row r="55" ht="25" customHeight="1">
+      <x:c r="A55" s="1"/>
+      <x:c r="B55" s="1"/>
+      <x:c r="C55" s="1"/>
+      <x:c r="D55" s="1"/>
+    </x:row>
+    <x:row r="56" ht="25" customHeight="1">
+      <x:c r="A56" s="1"/>
+      <x:c r="B56" s="1"/>
+      <x:c r="C56" s="1"/>
+      <x:c r="D56" s="1"/>
+    </x:row>
+    <x:row r="57" ht="30" customHeight="1">
+      <x:c r="A57" s="8" t="str">
+        <x:v>Contribution change by driver</x:v>
+      </x:c>
+      <x:c r="B57" s="8"/>
+      <x:c r="C57" s="8"/>
+      <x:c r="D57" s="1"/>
+    </x:row>
+    <x:row r="58" ht="25" customHeight="1">
+      <x:c r="A58" s="1" t="str">
+        <x:v>First-visit revenue</x:v>
+      </x:c>
+      <x:c r="B58" s="1"/>
+      <x:c r="C58" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C12-B12,"Complete both columns")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D58" s="1"/>
+    </x:row>
+    <x:row r="59" ht="25" customHeight="1">
+      <x:c r="A59" s="1" t="str">
+        <x:v>First-visit labour</x:v>
+      </x:c>
+      <x:c r="B59" s="1"/>
+      <x:c r="C59" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B22-C22,"Complete both columns")</x:f>
+        <x:v>-25</x:v>
+      </x:c>
+      <x:c r="D59" s="1"/>
+    </x:row>
+    <x:row r="60" ht="25" customHeight="1">
+      <x:c r="A60" s="1" t="str">
+        <x:v>First-visit supplies</x:v>
+      </x:c>
+      <x:c r="B60" s="1"/>
+      <x:c r="C60" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B15-C15,"Complete both columns")</x:f>
+        <x:v>-3</x:v>
+      </x:c>
+      <x:c r="D60" s="1"/>
+    </x:row>
+    <x:row r="61" ht="25" customHeight="1">
+      <x:c r="A61" s="1" t="str">
+        <x:v>First-visit travel</x:v>
+      </x:c>
+      <x:c r="B61" s="1"/>
+      <x:c r="C61" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B16-C16,"Complete both columns")</x:f>
+        <x:v>-4</x:v>
+      </x:c>
+      <x:c r="D61" s="1"/>
+    </x:row>
+    <x:row r="62" ht="25" customHeight="1">
+      <x:c r="A62" s="1" t="str">
+        <x:v>First-visit other direct costs</x:v>
+      </x:c>
+      <x:c r="B62" s="1"/>
+      <x:c r="C62" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B17-C17,"Complete both columns")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D62" s="1"/>
+    </x:row>
+    <x:row r="63" ht="25" customHeight="1">
+      <x:c r="A63" s="1" t="str">
+        <x:v>Payment fees</x:v>
+      </x:c>
+      <x:c r="B63" s="1"/>
+      <x:c r="C63" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B23-C23,"Complete both columns")</x:f>
+        <x:v>-8.881784197001252e-16</x:v>
+      </x:c>
+      <x:c r="D63" s="1"/>
+    </x:row>
+    <x:row r="64" ht="25" customHeight="1">
+      <x:c r="A64" s="1" t="str">
+        <x:v>Callback</x:v>
+      </x:c>
+      <x:c r="B64" s="1"/>
+      <x:c r="C64" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),-C48,"Complete both columns")</x:f>
+        <x:v>-37</x:v>
+      </x:c>
+      <x:c r="D64" s="1"/>
+    </x:row>
+    <x:row r="65" ht="25" customHeight="1">
+      <x:c r="A65" s="1" t="str">
+        <x:v>Customer credit</x:v>
+      </x:c>
+      <x:c r="B65" s="1"/>
+      <x:c r="C65" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),-C42,"Complete both columns")</x:f>
+        <x:v>-20</x:v>
+      </x:c>
+      <x:c r="D65" s="1"/>
+    </x:row>
+    <x:row r="66" ht="25" customHeight="1">
+      <x:c r="A66" s="1" t="str">
+        <x:v>Extra work net contribution</x:v>
+      </x:c>
+      <x:c r="B66" s="1"/>
+      <x:c r="C66" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C44-C45,"Complete both columns")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D66" s="1"/>
+    </x:row>
+    <x:row r="67" ht="25" customHeight="1">
+      <x:c r="A67" s="1" t="str">
+        <x:v>Total contribution change</x:v>
+      </x:c>
+      <x:c r="B67" s="1"/>
+      <x:c r="C67" s="6" t="n">
+        <x:f>IF(COUNT(C58:C66)=9,SUM(C58:C66),"Complete both columns")</x:f>
+        <x:v>-89</x:v>
+      </x:c>
+      <x:c r="D67" s="1"/>
+    </x:row>
+    <x:row r="68" ht="48" customHeight="1">
+      <x:c r="A68" s="19" t="str">
+        <x:v>Enter callback and extra costs only when absent from first-visit actuals. Credit reduces revenue once.</x:v>
+      </x:c>
+      <x:c r="B68" s="1"/>
+      <x:c r="C68" s="1"/>
+      <x:c r="D68" s="1"/>
+    </x:row>
+    <x:row r="69" ht="48" customHeight="1">
+      <x:c r="A69" s="19" t="str">
+        <x:v>Blank fee override uses first-visit revenue × rate. Include extra-work fees once in override or extra costs.</x:v>
+      </x:c>
+      <x:c r="B69" s="1"/>
+      <x:c r="C69" s="1"/>
+      <x:c r="D69" s="1"/>
+    </x:row>
+    <x:row r="70" ht="48" customHeight="1">
+      <x:c r="A70" s="19" t="str">
+        <x:v>All figures use one currency. Contribution excludes fixed overhead. Example is fictional.</x:v>
+      </x:c>
+      <x:c r="B70" s="1"/>
+      <x:c r="C70" s="1"/>
+      <x:c r="D70" s="1"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="D5:D5">
@@ -1039,7 +1728,7 @@
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="decimal" operator="between" sqref="B12:C17">
       <x:formula1>0</x:formula1>
       <x:formula2>1000000000</x:formula2>
@@ -1048,6 +1737,10 @@
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="C37:C45">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1000000000</x:formula2>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Improve cleaning worksheet and matching guide [skip social]
Add callback/credit reconciliation and update existing resource and guide. User authorized release; tests, build, workbook checks and route audit passed. [skip social]
</commit_message>
<xml_diff>
--- a/public/downloads/mybreakeven-cleaning-job-cost.xlsx
+++ b/public/downloads/mybreakeven-cleaning-job-cost.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job" sheetId="1" r:id="R5b2f3fcdc73e4ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="2" r:id="Rae68ff4fac524359"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job" sheetId="1" r:id="R0ac3e104fdd3472d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="2" r:id="Rf406422c6b014f6e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -99,7 +99,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -115,6 +115,17 @@
     <x:xf numFmtId="202" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -361,7 +372,7 @@
     </x:row>
     <x:row r="3" ht="31" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Enter every input, including zero when a cost does not apply</x:v>
+        <x:v>Enter first-visit actuals; add adjustments below</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -381,19 +392,19 @@
         <x:v>Actual minus estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="1" t="str">
+    <x:row r="5" ht="48" customHeight="1">
+      <x:c r="A5" s="15" t="str">
         <x:v>Contribution before monthly overhead</x:v>
       </x:c>
-      <x:c r="B5" s="6" t="str">
+      <x:c r="B5" s="16" t="str">
         <x:f>B26</x:f>
         <x:v>Enter all inputs</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="str">
-        <x:f>C26</x:f>
-        <x:v>Enter all inputs</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="str">
+      <x:c r="C5" s="16" t="str">
+        <x:f>C51</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="str">
         <x:f>IF(AND(ISNUMBER(B5),ISNUMBER(C5)),C5-B5,"Complete both columns")</x:f>
         <x:v>Complete both columns</x:v>
       </x:c>
@@ -406,7 +417,7 @@
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="1" t="str">
-        <x:v>A lower contribution difference means less left for overhead.</x:v>
+        <x:v>Actual result includes adjustments below; costs entered once.</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -551,7 +562,7 @@
         <x:v>Enter all inputs</x:v>
       </x:c>
       <x:c r="C23" s="6" t="str">
-        <x:f>IF(COUNT(C12:C18)=7,C12*C18,"Enter all inputs")</x:f>
+        <x:f>IF(COUNT(C12:C18)=7,IF(ISNUMBER(C43),C43,C12*C18),"Enter all inputs")</x:f>
         <x:v>Enter all inputs</x:v>
       </x:c>
       <x:c r="D23" s="1"/>
@@ -652,11 +663,347 @@
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>Example source: MyBreakeven illustrative assumptions, October 10, 2026.</x:v>
+        <x:v>Example source: MyBreakeven illustrative assumptions, October 14, 2026.</x:v>
       </x:c>
       <x:c r="B34" s="14"/>
       <x:c r="C34" s="14"/>
       <x:c r="D34" s="14"/>
+    </x:row>
+    <x:row r="36" ht="30" customHeight="1">
+      <x:c r="A36" s="8" t="str">
+        <x:v>Additional actual job entries</x:v>
+      </x:c>
+      <x:c r="B36" s="8"/>
+      <x:c r="C36" s="8"/>
+      <x:c r="D36" s="1"/>
+    </x:row>
+    <x:row r="37" ht="25" customHeight="1">
+      <x:c r="A37" s="1" t="str">
+        <x:v>Callback paid crew-hours</x:v>
+      </x:c>
+      <x:c r="B37" s="1"/>
+      <x:c r="C37" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D37" s="1"/>
+    </x:row>
+    <x:row r="38" ht="25" customHeight="1">
+      <x:c r="A38" s="1" t="str">
+        <x:v>Callback loaded cost per crew-hour</x:v>
+      </x:c>
+      <x:c r="B38" s="1"/>
+      <x:c r="C38" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="25" customHeight="1">
+      <x:c r="A39" s="1" t="str">
+        <x:v>Callback supplies</x:v>
+      </x:c>
+      <x:c r="B39" s="1"/>
+      <x:c r="C39" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="25" customHeight="1">
+      <x:c r="A40" s="1" t="str">
+        <x:v>Callback travel</x:v>
+      </x:c>
+      <x:c r="B40" s="1"/>
+      <x:c r="C40" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="25" customHeight="1">
+      <x:c r="A41" s="1" t="str">
+        <x:v>Callback other direct costs</x:v>
+      </x:c>
+      <x:c r="B41" s="1"/>
+      <x:c r="C41" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="25" customHeight="1">
+      <x:c r="A42" s="1" t="str">
+        <x:v>Customer credit / revenue reduction</x:v>
+      </x:c>
+      <x:c r="B42" s="1"/>
+      <x:c r="C42" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="25" customHeight="1">
+      <x:c r="A43" s="1" t="str">
+        <x:v>Actual payment fees (optional override)</x:v>
+      </x:c>
+      <x:c r="B43" s="1"/>
+      <x:c r="C43" s="11"/>
+      <x:c r="D43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="25" customHeight="1">
+      <x:c r="A44" s="1" t="str">
+        <x:v>Extra work revenue</x:v>
+      </x:c>
+      <x:c r="B44" s="1"/>
+      <x:c r="C44" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D44" s="1"/>
+    </x:row>
+    <x:row r="45" ht="25" customHeight="1">
+      <x:c r="A45" s="1" t="str">
+        <x:v>Extra work variable costs</x:v>
+      </x:c>
+      <x:c r="B45" s="1"/>
+      <x:c r="C45" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D45" s="1"/>
+    </x:row>
+    <x:row r="46" ht="25" customHeight="1">
+      <x:c r="A46" s="1"/>
+      <x:c r="B46" s="1"/>
+      <x:c r="C46" s="1"/>
+      <x:c r="D46" s="1"/>
+    </x:row>
+    <x:row r="47" ht="30" customHeight="1">
+      <x:c r="A47" s="8" t="str">
+        <x:v>Final job result</x:v>
+      </x:c>
+      <x:c r="B47" s="8"/>
+      <x:c r="C47" s="8"/>
+      <x:c r="D47" s="1"/>
+    </x:row>
+    <x:row r="48" ht="25" customHeight="1">
+      <x:c r="A48" s="1" t="str">
+        <x:v>Callback cost</x:v>
+      </x:c>
+      <x:c r="B48" s="1"/>
+      <x:c r="C48" s="6" t="n">
+        <x:f>IF(COUNT(C37:C42,C44:C45)=8,C37*C38+SUM(C39:C41),"Enter every adjustment")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D48" s="1"/>
+    </x:row>
+    <x:row r="49" ht="25" customHeight="1">
+      <x:c r="A49" s="1" t="str">
+        <x:v>Final retained revenue</x:v>
+      </x:c>
+      <x:c r="B49" s="1"/>
+      <x:c r="C49" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(C26),ISNUMBER(C48)),C12-C42+C44,"Complete actual and adjustments")</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D49" s="1"/>
+    </x:row>
+    <x:row r="50" ht="25" customHeight="1">
+      <x:c r="A50" s="1" t="str">
+        <x:v>Total variable costs incl. adjustments</x:v>
+      </x:c>
+      <x:c r="B50" s="1"/>
+      <x:c r="C50" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(C24),ISNUMBER(C48)),C24+C48+C45,"Complete actual and adjustments")</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D50" s="1"/>
+    </x:row>
+    <x:row r="51" ht="25" customHeight="1">
+      <x:c r="A51" s="1" t="str">
+        <x:v>Final contribution before overhead</x:v>
+      </x:c>
+      <x:c r="B51" s="1"/>
+      <x:c r="C51" s="17" t="str">
+        <x:f>IF(AND(ISNUMBER(C49),ISNUMBER(C50)),C49-C50,"Complete actual and adjustments")</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D51" s="1"/>
+    </x:row>
+    <x:row r="52" ht="25" customHeight="1">
+      <x:c r="A52" s="1" t="str">
+        <x:v>Contribution / retained revenue</x:v>
+      </x:c>
+      <x:c r="B52" s="1"/>
+      <x:c r="C52" s="18" t="str">
+        <x:f>IF(AND(ISNUMBER(C51),ISNUMBER(C49)),IF(C49=0,"n.a.",C51/C49),"Complete actual and adjustments")</x:f>
+        <x:v>Complete actual and adjustments</x:v>
+      </x:c>
+      <x:c r="D52" s="1"/>
+    </x:row>
+    <x:row r="53" ht="25" customHeight="1">
+      <x:c r="A53" s="1" t="str">
+        <x:v>Final actual minus estimate</x:v>
+      </x:c>
+      <x:c r="B53" s="1"/>
+      <x:c r="C53" s="17" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C51-B26,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D53" s="1"/>
+    </x:row>
+    <x:row r="54" ht="25" customHeight="1">
+      <x:c r="A54" s="1"/>
+      <x:c r="B54" s="1"/>
+      <x:c r="C54" s="1"/>
+      <x:c r="D54" s="1"/>
+    </x:row>
+    <x:row r="55" ht="25" customHeight="1">
+      <x:c r="A55" s="1"/>
+      <x:c r="B55" s="1"/>
+      <x:c r="C55" s="1"/>
+      <x:c r="D55" s="1"/>
+    </x:row>
+    <x:row r="56" ht="25" customHeight="1">
+      <x:c r="A56" s="1"/>
+      <x:c r="B56" s="1"/>
+      <x:c r="C56" s="1"/>
+      <x:c r="D56" s="1"/>
+    </x:row>
+    <x:row r="57" ht="30" customHeight="1">
+      <x:c r="A57" s="8" t="str">
+        <x:v>Contribution change by driver</x:v>
+      </x:c>
+      <x:c r="B57" s="8"/>
+      <x:c r="C57" s="8"/>
+      <x:c r="D57" s="1"/>
+    </x:row>
+    <x:row r="58" ht="25" customHeight="1">
+      <x:c r="A58" s="1" t="str">
+        <x:v>First-visit revenue</x:v>
+      </x:c>
+      <x:c r="B58" s="1"/>
+      <x:c r="C58" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C12-B12,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D58" s="1"/>
+    </x:row>
+    <x:row r="59" ht="25" customHeight="1">
+      <x:c r="A59" s="1" t="str">
+        <x:v>First-visit labour</x:v>
+      </x:c>
+      <x:c r="B59" s="1"/>
+      <x:c r="C59" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B22-C22,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D59" s="1"/>
+    </x:row>
+    <x:row r="60" ht="25" customHeight="1">
+      <x:c r="A60" s="1" t="str">
+        <x:v>First-visit supplies</x:v>
+      </x:c>
+      <x:c r="B60" s="1"/>
+      <x:c r="C60" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B15-C15,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D60" s="1"/>
+    </x:row>
+    <x:row r="61" ht="25" customHeight="1">
+      <x:c r="A61" s="1" t="str">
+        <x:v>First-visit travel</x:v>
+      </x:c>
+      <x:c r="B61" s="1"/>
+      <x:c r="C61" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B16-C16,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D61" s="1"/>
+    </x:row>
+    <x:row r="62" ht="25" customHeight="1">
+      <x:c r="A62" s="1" t="str">
+        <x:v>First-visit other direct costs</x:v>
+      </x:c>
+      <x:c r="B62" s="1"/>
+      <x:c r="C62" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B17-C17,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D62" s="1"/>
+    </x:row>
+    <x:row r="63" ht="25" customHeight="1">
+      <x:c r="A63" s="1" t="str">
+        <x:v>Payment fees</x:v>
+      </x:c>
+      <x:c r="B63" s="1"/>
+      <x:c r="C63" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B23-C23,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D63" s="1"/>
+    </x:row>
+    <x:row r="64" ht="25" customHeight="1">
+      <x:c r="A64" s="1" t="str">
+        <x:v>Callback</x:v>
+      </x:c>
+      <x:c r="B64" s="1"/>
+      <x:c r="C64" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),-C48,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D64" s="1"/>
+    </x:row>
+    <x:row r="65" ht="25" customHeight="1">
+      <x:c r="A65" s="1" t="str">
+        <x:v>Customer credit</x:v>
+      </x:c>
+      <x:c r="B65" s="1"/>
+      <x:c r="C65" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),-C42,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D65" s="1"/>
+    </x:row>
+    <x:row r="66" ht="25" customHeight="1">
+      <x:c r="A66" s="1" t="str">
+        <x:v>Extra work net contribution</x:v>
+      </x:c>
+      <x:c r="B66" s="1"/>
+      <x:c r="C66" s="6" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C44-C45,"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D66" s="1"/>
+    </x:row>
+    <x:row r="67" ht="25" customHeight="1">
+      <x:c r="A67" s="1" t="str">
+        <x:v>Total contribution change</x:v>
+      </x:c>
+      <x:c r="B67" s="1"/>
+      <x:c r="C67" s="6" t="str">
+        <x:f>IF(COUNT(C58:C66)=9,SUM(C58:C66),"Complete both columns")</x:f>
+        <x:v>Complete both columns</x:v>
+      </x:c>
+      <x:c r="D67" s="1"/>
+    </x:row>
+    <x:row r="68" ht="48" customHeight="1">
+      <x:c r="A68" s="19" t="str">
+        <x:v>Enter callback and extra costs only when absent from first-visit actuals. Credit reduces revenue once.</x:v>
+      </x:c>
+      <x:c r="B68" s="1"/>
+      <x:c r="C68" s="1"/>
+      <x:c r="D68" s="1"/>
+    </x:row>
+    <x:row r="69" ht="48" customHeight="1">
+      <x:c r="A69" s="19" t="str">
+        <x:v>Blank fee override uses first-visit revenue × rate. Include extra-work fees once in override or extra costs.</x:v>
+      </x:c>
+      <x:c r="B69" s="1"/>
+      <x:c r="C69" s="1"/>
+      <x:c r="D69" s="1"/>
+    </x:row>
+    <x:row r="70" ht="48" customHeight="1">
+      <x:c r="A70" s="19" t="str">
+        <x:v>All figures use one currency. Contribution excludes fixed overhead. Example is fictional.</x:v>
+      </x:c>
+      <x:c r="B70" s="1"/>
+      <x:c r="C70" s="1"/>
+      <x:c r="D70" s="1"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="D5:D5">
@@ -664,7 +1011,7 @@
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="decimal" operator="between" sqref="B12:C17">
       <x:formula1>0</x:formula1>
       <x:formula2>1000000000</x:formula2>
@@ -672,6 +1019,10 @@
     <x:dataValidation type="decimal" operator="between" sqref="B18:C18">
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="C37:C45">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1000000000</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -704,7 +1055,7 @@
     </x:row>
     <x:row r="3" ht="31" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Illustrative USD example, not a customer result</x:v>
+        <x:v>Fictional USD job including callback and credit</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -724,21 +1075,21 @@
         <x:v>Actual minus estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="1" t="str">
+    <x:row r="5" ht="48" customHeight="1">
+      <x:c r="A5" s="15" t="str">
         <x:v>Contribution before monthly overhead</x:v>
       </x:c>
-      <x:c r="B5" s="6" t="n">
+      <x:c r="B5" s="16" t="n">
         <x:f>B26</x:f>
         <x:v>110.80000000000001</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="n">
-        <x:f>C26</x:f>
-        <x:v>78.80000000000001</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="n">
+      <x:c r="C5" s="16" t="n">
+        <x:f>C51</x:f>
+        <x:v>21.80000000000001</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="n">
         <x:f>IF(AND(ISNUMBER(B5),ISNUMBER(C5)),C5-B5,"Complete both columns")</x:f>
-        <x:v>-32</x:v>
+        <x:v>-89</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
@@ -749,7 +1100,7 @@
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="1" t="str">
-        <x:v>A lower contribution difference means less left for overhead.</x:v>
+        <x:v>Actual result includes adjustments below; costs entered once.</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -926,8 +1277,8 @@
         <x:v>7.199999999999999</x:v>
       </x:c>
       <x:c r="C23" s="6" t="n">
-        <x:f>IF(COUNT(C12:C18)=7,C12*C18,"Enter all inputs")</x:f>
-        <x:v>7.199999999999999</x:v>
+        <x:f>IF(COUNT(C12:C18)=7,IF(ISNUMBER(C43),C43,C12*C18),"Enter all inputs")</x:f>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="D23" s="1"/>
     </x:row>
@@ -1027,11 +1378,349 @@
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>Example source: MyBreakeven illustrative assumptions, October 10, 2026.</x:v>
+        <x:v>Example source: MyBreakeven illustrative assumptions, October 14, 2026.</x:v>
       </x:c>
       <x:c r="B34" s="14"/>
       <x:c r="C34" s="14"/>
       <x:c r="D34" s="14"/>
+    </x:row>
+    <x:row r="36" ht="30" customHeight="1">
+      <x:c r="A36" s="8" t="str">
+        <x:v>Additional actual job entries</x:v>
+      </x:c>
+      <x:c r="B36" s="8"/>
+      <x:c r="C36" s="8"/>
+      <x:c r="D36" s="1"/>
+    </x:row>
+    <x:row r="37" ht="25" customHeight="1">
+      <x:c r="A37" s="1" t="str">
+        <x:v>Callback paid crew-hours</x:v>
+      </x:c>
+      <x:c r="B37" s="1"/>
+      <x:c r="C37" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D37" s="1"/>
+    </x:row>
+    <x:row r="38" ht="25" customHeight="1">
+      <x:c r="A38" s="1" t="str">
+        <x:v>Callback loaded cost per crew-hour</x:v>
+      </x:c>
+      <x:c r="B38" s="1"/>
+      <x:c r="C38" s="11" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="25" customHeight="1">
+      <x:c r="A39" s="1" t="str">
+        <x:v>Callback supplies</x:v>
+      </x:c>
+      <x:c r="B39" s="1"/>
+      <x:c r="C39" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="25" customHeight="1">
+      <x:c r="A40" s="1" t="str">
+        <x:v>Callback travel</x:v>
+      </x:c>
+      <x:c r="B40" s="1"/>
+      <x:c r="C40" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="25" customHeight="1">
+      <x:c r="A41" s="1" t="str">
+        <x:v>Callback other direct costs</x:v>
+      </x:c>
+      <x:c r="B41" s="1"/>
+      <x:c r="C41" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="25" customHeight="1">
+      <x:c r="A42" s="1" t="str">
+        <x:v>Customer credit / revenue reduction</x:v>
+      </x:c>
+      <x:c r="B42" s="1"/>
+      <x:c r="C42" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="25" customHeight="1">
+      <x:c r="A43" s="1" t="str">
+        <x:v>Actual payment fees (optional override)</x:v>
+      </x:c>
+      <x:c r="B43" s="1"/>
+      <x:c r="C43" s="11" t="n">
+        <x:v>7.2</x:v>
+      </x:c>
+      <x:c r="D43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="25" customHeight="1">
+      <x:c r="A44" s="1" t="str">
+        <x:v>Extra work revenue</x:v>
+      </x:c>
+      <x:c r="B44" s="1"/>
+      <x:c r="C44" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D44" s="1"/>
+    </x:row>
+    <x:row r="45" ht="25" customHeight="1">
+      <x:c r="A45" s="1" t="str">
+        <x:v>Extra work variable costs</x:v>
+      </x:c>
+      <x:c r="B45" s="1"/>
+      <x:c r="C45" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D45" s="1"/>
+    </x:row>
+    <x:row r="46" ht="25" customHeight="1">
+      <x:c r="A46" s="1"/>
+      <x:c r="B46" s="1"/>
+      <x:c r="C46" s="1"/>
+      <x:c r="D46" s="1"/>
+    </x:row>
+    <x:row r="47" ht="30" customHeight="1">
+      <x:c r="A47" s="8" t="str">
+        <x:v>Final job result</x:v>
+      </x:c>
+      <x:c r="B47" s="8"/>
+      <x:c r="C47" s="8"/>
+      <x:c r="D47" s="1"/>
+    </x:row>
+    <x:row r="48" ht="25" customHeight="1">
+      <x:c r="A48" s="1" t="str">
+        <x:v>Callback cost</x:v>
+      </x:c>
+      <x:c r="B48" s="1"/>
+      <x:c r="C48" s="6" t="n">
+        <x:f>IF(COUNT(C37:C42,C44:C45)=8,C37*C38+SUM(C39:C41),"Enter every adjustment")</x:f>
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="D48" s="1"/>
+    </x:row>
+    <x:row r="49" ht="25" customHeight="1">
+      <x:c r="A49" s="1" t="str">
+        <x:v>Final retained revenue</x:v>
+      </x:c>
+      <x:c r="B49" s="1"/>
+      <x:c r="C49" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(C26),ISNUMBER(C48)),C12-C42+C44,"Complete actual and adjustments")</x:f>
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="D49" s="1"/>
+    </x:row>
+    <x:row r="50" ht="25" customHeight="1">
+      <x:c r="A50" s="1" t="str">
+        <x:v>Total variable costs incl. adjustments</x:v>
+      </x:c>
+      <x:c r="B50" s="1"/>
+      <x:c r="C50" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(C24),ISNUMBER(C48)),C24+C48+C45,"Complete actual and adjustments")</x:f>
+        <x:v>198.2</x:v>
+      </x:c>
+      <x:c r="D50" s="1"/>
+    </x:row>
+    <x:row r="51" ht="25" customHeight="1">
+      <x:c r="A51" s="1" t="str">
+        <x:v>Final contribution before overhead</x:v>
+      </x:c>
+      <x:c r="B51" s="1"/>
+      <x:c r="C51" s="17" t="n">
+        <x:f>IF(AND(ISNUMBER(C49),ISNUMBER(C50)),C49-C50,"Complete actual and adjustments")</x:f>
+        <x:v>21.80000000000001</x:v>
+      </x:c>
+      <x:c r="D51" s="1"/>
+    </x:row>
+    <x:row r="52" ht="25" customHeight="1">
+      <x:c r="A52" s="1" t="str">
+        <x:v>Contribution / retained revenue</x:v>
+      </x:c>
+      <x:c r="B52" s="1"/>
+      <x:c r="C52" s="18" t="n">
+        <x:f>IF(AND(ISNUMBER(C51),ISNUMBER(C49)),IF(C49=0,"n.a.",C51/C49),"Complete actual and adjustments")</x:f>
+        <x:v>0.09909090909090915</x:v>
+      </x:c>
+      <x:c r="D52" s="1"/>
+    </x:row>
+    <x:row r="53" ht="25" customHeight="1">
+      <x:c r="A53" s="1" t="str">
+        <x:v>Final actual minus estimate</x:v>
+      </x:c>
+      <x:c r="B53" s="1"/>
+      <x:c r="C53" s="17" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C51-B26,"Complete both columns")</x:f>
+        <x:v>-89</x:v>
+      </x:c>
+      <x:c r="D53" s="1"/>
+    </x:row>
+    <x:row r="54" ht="25" customHeight="1">
+      <x:c r="A54" s="1"/>
+      <x:c r="B54" s="1"/>
+      <x:c r="C54" s="1"/>
+      <x:c r="D54" s="1"/>
+    </x:row>
+    <x:row r="55" ht="25" customHeight="1">
+      <x:c r="A55" s="1"/>
+      <x:c r="B55" s="1"/>
+      <x:c r="C55" s="1"/>
+      <x:c r="D55" s="1"/>
+    </x:row>
+    <x:row r="56" ht="25" customHeight="1">
+      <x:c r="A56" s="1"/>
+      <x:c r="B56" s="1"/>
+      <x:c r="C56" s="1"/>
+      <x:c r="D56" s="1"/>
+    </x:row>
+    <x:row r="57" ht="30" customHeight="1">
+      <x:c r="A57" s="8" t="str">
+        <x:v>Contribution change by driver</x:v>
+      </x:c>
+      <x:c r="B57" s="8"/>
+      <x:c r="C57" s="8"/>
+      <x:c r="D57" s="1"/>
+    </x:row>
+    <x:row r="58" ht="25" customHeight="1">
+      <x:c r="A58" s="1" t="str">
+        <x:v>First-visit revenue</x:v>
+      </x:c>
+      <x:c r="B58" s="1"/>
+      <x:c r="C58" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C12-B12,"Complete both columns")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D58" s="1"/>
+    </x:row>
+    <x:row r="59" ht="25" customHeight="1">
+      <x:c r="A59" s="1" t="str">
+        <x:v>First-visit labour</x:v>
+      </x:c>
+      <x:c r="B59" s="1"/>
+      <x:c r="C59" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B22-C22,"Complete both columns")</x:f>
+        <x:v>-25</x:v>
+      </x:c>
+      <x:c r="D59" s="1"/>
+    </x:row>
+    <x:row r="60" ht="25" customHeight="1">
+      <x:c r="A60" s="1" t="str">
+        <x:v>First-visit supplies</x:v>
+      </x:c>
+      <x:c r="B60" s="1"/>
+      <x:c r="C60" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B15-C15,"Complete both columns")</x:f>
+        <x:v>-3</x:v>
+      </x:c>
+      <x:c r="D60" s="1"/>
+    </x:row>
+    <x:row r="61" ht="25" customHeight="1">
+      <x:c r="A61" s="1" t="str">
+        <x:v>First-visit travel</x:v>
+      </x:c>
+      <x:c r="B61" s="1"/>
+      <x:c r="C61" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B16-C16,"Complete both columns")</x:f>
+        <x:v>-4</x:v>
+      </x:c>
+      <x:c r="D61" s="1"/>
+    </x:row>
+    <x:row r="62" ht="25" customHeight="1">
+      <x:c r="A62" s="1" t="str">
+        <x:v>First-visit other direct costs</x:v>
+      </x:c>
+      <x:c r="B62" s="1"/>
+      <x:c r="C62" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B17-C17,"Complete both columns")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D62" s="1"/>
+    </x:row>
+    <x:row r="63" ht="25" customHeight="1">
+      <x:c r="A63" s="1" t="str">
+        <x:v>Payment fees</x:v>
+      </x:c>
+      <x:c r="B63" s="1"/>
+      <x:c r="C63" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),B23-C23,"Complete both columns")</x:f>
+        <x:v>-8.881784197001252e-16</x:v>
+      </x:c>
+      <x:c r="D63" s="1"/>
+    </x:row>
+    <x:row r="64" ht="25" customHeight="1">
+      <x:c r="A64" s="1" t="str">
+        <x:v>Callback</x:v>
+      </x:c>
+      <x:c r="B64" s="1"/>
+      <x:c r="C64" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),-C48,"Complete both columns")</x:f>
+        <x:v>-37</x:v>
+      </x:c>
+      <x:c r="D64" s="1"/>
+    </x:row>
+    <x:row r="65" ht="25" customHeight="1">
+      <x:c r="A65" s="1" t="str">
+        <x:v>Customer credit</x:v>
+      </x:c>
+      <x:c r="B65" s="1"/>
+      <x:c r="C65" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),-C42,"Complete both columns")</x:f>
+        <x:v>-20</x:v>
+      </x:c>
+      <x:c r="D65" s="1"/>
+    </x:row>
+    <x:row r="66" ht="25" customHeight="1">
+      <x:c r="A66" s="1" t="str">
+        <x:v>Extra work net contribution</x:v>
+      </x:c>
+      <x:c r="B66" s="1"/>
+      <x:c r="C66" s="6" t="n">
+        <x:f>IF(AND(ISNUMBER(B26),ISNUMBER(C51)),C44-C45,"Complete both columns")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D66" s="1"/>
+    </x:row>
+    <x:row r="67" ht="25" customHeight="1">
+      <x:c r="A67" s="1" t="str">
+        <x:v>Total contribution change</x:v>
+      </x:c>
+      <x:c r="B67" s="1"/>
+      <x:c r="C67" s="6" t="n">
+        <x:f>IF(COUNT(C58:C66)=9,SUM(C58:C66),"Complete both columns")</x:f>
+        <x:v>-89</x:v>
+      </x:c>
+      <x:c r="D67" s="1"/>
+    </x:row>
+    <x:row r="68" ht="48" customHeight="1">
+      <x:c r="A68" s="19" t="str">
+        <x:v>Enter callback and extra costs only when absent from first-visit actuals. Credit reduces revenue once.</x:v>
+      </x:c>
+      <x:c r="B68" s="1"/>
+      <x:c r="C68" s="1"/>
+      <x:c r="D68" s="1"/>
+    </x:row>
+    <x:row r="69" ht="48" customHeight="1">
+      <x:c r="A69" s="19" t="str">
+        <x:v>Blank fee override uses first-visit revenue × rate. Include extra-work fees once in override or extra costs.</x:v>
+      </x:c>
+      <x:c r="B69" s="1"/>
+      <x:c r="C69" s="1"/>
+      <x:c r="D69" s="1"/>
+    </x:row>
+    <x:row r="70" ht="48" customHeight="1">
+      <x:c r="A70" s="19" t="str">
+        <x:v>All figures use one currency. Contribution excludes fixed overhead. Example is fictional.</x:v>
+      </x:c>
+      <x:c r="B70" s="1"/>
+      <x:c r="C70" s="1"/>
+      <x:c r="D70" s="1"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="D5:D5">
@@ -1039,7 +1728,7 @@
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="decimal" operator="between" sqref="B12:C17">
       <x:formula1>0</x:formula1>
       <x:formula2>1000000000</x:formula2>
@@ -1048,6 +1737,10 @@
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="C37:C45">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1000000000</x:formula2>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>